<commit_message>
Add Monster brand simulator with shared multi-brand Streamlit app
Combined Coca-Cola and Monster into a single app with sidebar brand selector.
Added month picker, 5 reward tiers, Monster SKU editor with Size column,
store penetration from raw order data, and CSV/Excel import for proposed points.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/M-rewards-cocacola.xlsx
+++ b/M-rewards-cocacola.xlsx
@@ -5,24 +5,24 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rickrangel/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rickrangel/mercaso-concierge/sso/M-Rewards/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBDF4D81-AA26-C348-BE3D-86E1FE6383DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8DCB4C-720C-3E4E-94AE-DE26A884C346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Claude Log" sheetId="5" r:id="rId1"/>
     <sheet name="ims" sheetId="1" r:id="rId2"/>
     <sheet name="coca-cola-rewards" sheetId="2" r:id="rId3"/>
-    <sheet name="WOS Ranked" sheetId="4" r:id="rId4"/>
+    <sheet name="sku's-coca-cola" sheetId="4" r:id="rId4"/>
     <sheet name="rewards" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'coca-cola-rewards'!$A$1:$D$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">ims!$A$1:$BK$269</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'WOS Ranked'!$A$1:$O$269</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'sku''s-coca-cola'!$A$1:$O$269</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>

<commit_message>
Add editable reward thresholds and update Coca-Cola workbook
Reward tiers can now be added/removed per brand in the UI; Ferrera
defaults corrected to its own 3 tiers (5000/10000/15000).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/M-rewards-cocacola.xlsx
+++ b/M-rewards-cocacola.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rickrangel/mercaso-concierge/sso/M-Rewards/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8DCB4C-720C-3E4E-94AE-DE26A884C346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F6BA402-47BE-FD46-9C38-A5369CA8969A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55447,6 +55447,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A28DBFC5-8611-0B45-8E7C-1B1F27A6DFE8}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:O279"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
@@ -55511,7 +55512,7 @@
         <v>2600</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" hidden="1">
       <c r="A2" s="44">
         <v>1</v>
       </c>
@@ -55549,7 +55550,7 @@
       <c r="N2" s="29"/>
       <c r="O2" s="48"/>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" hidden="1">
       <c r="A3" s="44">
         <v>2</v>
       </c>
@@ -55587,7 +55588,7 @@
       <c r="N3" s="29"/>
       <c r="O3" s="48"/>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" hidden="1">
       <c r="A4" s="44">
         <v>3</v>
       </c>
@@ -55625,7 +55626,7 @@
       <c r="N4" s="29"/>
       <c r="O4" s="48"/>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" hidden="1">
       <c r="A5" s="44">
         <v>4</v>
       </c>
@@ -55663,7 +55664,7 @@
       <c r="N5" s="29"/>
       <c r="O5" s="48"/>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" hidden="1">
       <c r="A6" s="44">
         <v>5</v>
       </c>
@@ -55701,7 +55702,7 @@
       <c r="N6" s="29"/>
       <c r="O6" s="48"/>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" hidden="1">
       <c r="A7" s="44">
         <v>6</v>
       </c>
@@ -55739,7 +55740,7 @@
       <c r="N7" s="29"/>
       <c r="O7" s="48"/>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" hidden="1">
       <c r="A8" s="44">
         <v>7</v>
       </c>
@@ -55825,7 +55826,7 @@
         <v>8616233800</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" hidden="1">
       <c r="A10" s="44">
         <v>9</v>
       </c>
@@ -55911,7 +55912,7 @@
         <v>4900004086</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" hidden="1">
       <c r="A12" s="44">
         <v>11</v>
       </c>
@@ -55949,7 +55950,7 @@
       <c r="N12" s="29"/>
       <c r="O12" s="53"/>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" hidden="1">
       <c r="A13" s="44">
         <v>12</v>
       </c>
@@ -55987,7 +55988,7 @@
       <c r="N13" s="29"/>
       <c r="O13" s="53"/>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" hidden="1">
       <c r="A14" s="44">
         <v>13</v>
       </c>
@@ -56121,7 +56122,7 @@
         <v>8616201000</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:15" hidden="1">
       <c r="A17" s="44">
         <v>16</v>
       </c>
@@ -56159,7 +56160,7 @@
       <c r="N17" s="29"/>
       <c r="O17" s="53"/>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:15" hidden="1">
       <c r="A18" s="44">
         <v>17</v>
       </c>
@@ -56245,7 +56246,7 @@
         <v>8616208000</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
+    <row r="20" spans="1:15" hidden="1">
       <c r="A20" s="44">
         <v>19</v>
       </c>
@@ -56283,7 +56284,7 @@
       <c r="N20" s="29"/>
       <c r="O20" s="53"/>
     </row>
-    <row r="21" spans="1:15">
+    <row r="21" spans="1:15" hidden="1">
       <c r="A21" s="44">
         <v>20</v>
       </c>
@@ -56321,7 +56322,7 @@
       <c r="N21" s="29"/>
       <c r="O21" s="53"/>
     </row>
-    <row r="22" spans="1:15">
+    <row r="22" spans="1:15" hidden="1">
       <c r="A22" s="44">
         <v>21</v>
       </c>
@@ -56359,7 +56360,7 @@
       <c r="N22" s="29"/>
       <c r="O22" s="53"/>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" spans="1:15" hidden="1">
       <c r="A23" s="44">
         <v>22</v>
       </c>
@@ -56397,7 +56398,7 @@
       <c r="N23" s="29"/>
       <c r="O23" s="53"/>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" spans="1:15" hidden="1">
       <c r="A24" s="44">
         <v>23</v>
       </c>
@@ -56435,7 +56436,7 @@
       <c r="N24" s="29"/>
       <c r="O24" s="53"/>
     </row>
-    <row r="25" spans="1:15">
+    <row r="25" spans="1:15" hidden="1">
       <c r="A25" s="44">
         <v>24</v>
       </c>
@@ -56473,7 +56474,7 @@
       <c r="N25" s="29"/>
       <c r="O25" s="53"/>
     </row>
-    <row r="26" spans="1:15">
+    <row r="26" spans="1:15" hidden="1">
       <c r="A26" s="44">
         <v>25</v>
       </c>
@@ -56511,7 +56512,7 @@
       <c r="N26" s="29"/>
       <c r="O26" s="53"/>
     </row>
-    <row r="27" spans="1:15">
+    <row r="27" spans="1:15" hidden="1">
       <c r="A27" s="44">
         <v>26</v>
       </c>
@@ -56597,7 +56598,7 @@
         <v>8616241116</v>
       </c>
     </row>
-    <row r="29" spans="1:15">
+    <row r="29" spans="1:15" hidden="1">
       <c r="A29" s="44">
         <v>28</v>
       </c>
@@ -56635,7 +56636,7 @@
       <c r="N29" s="29"/>
       <c r="O29" s="53"/>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" spans="1:15" hidden="1">
       <c r="A30" s="44">
         <v>29</v>
       </c>
@@ -56673,7 +56674,7 @@
       <c r="N30" s="29"/>
       <c r="O30" s="53"/>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" spans="1:15" hidden="1">
       <c r="A31" s="44">
         <v>30</v>
       </c>
@@ -56759,7 +56760,7 @@
         <v>8616220043</v>
       </c>
     </row>
-    <row r="33" spans="1:15">
+    <row r="33" spans="1:15" hidden="1">
       <c r="A33" s="44">
         <v>32</v>
       </c>
@@ -56797,7 +56798,7 @@
       <c r="N33" s="29"/>
       <c r="O33" s="53"/>
     </row>
-    <row r="34" spans="1:15">
+    <row r="34" spans="1:15" hidden="1">
       <c r="A34" s="44">
         <v>33</v>
       </c>
@@ -56835,7 +56836,7 @@
       <c r="N34" s="29"/>
       <c r="O34" s="53"/>
     </row>
-    <row r="35" spans="1:15">
+    <row r="35" spans="1:15" hidden="1">
       <c r="A35" s="44">
         <v>34</v>
       </c>
@@ -56873,7 +56874,7 @@
       <c r="N35" s="29"/>
       <c r="O35" s="53"/>
     </row>
-    <row r="36" spans="1:15">
+    <row r="36" spans="1:15" hidden="1">
       <c r="A36" s="44">
         <v>35</v>
       </c>
@@ -56911,7 +56912,7 @@
       <c r="N36" s="29"/>
       <c r="O36" s="53"/>
     </row>
-    <row r="37" spans="1:15">
+    <row r="37" spans="1:15" hidden="1">
       <c r="A37" s="44">
         <v>36</v>
       </c>
@@ -56949,7 +56950,7 @@
       <c r="N37" s="29"/>
       <c r="O37" s="53"/>
     </row>
-    <row r="38" spans="1:15">
+    <row r="38" spans="1:15" hidden="1">
       <c r="A38" s="44">
         <v>37</v>
       </c>
@@ -56987,7 +56988,7 @@
       <c r="N38" s="29"/>
       <c r="O38" s="53"/>
     </row>
-    <row r="39" spans="1:15">
+    <row r="39" spans="1:15" hidden="1">
       <c r="A39" s="44">
         <v>38</v>
       </c>
@@ -57025,7 +57026,7 @@
       <c r="N39" s="29"/>
       <c r="O39" s="53"/>
     </row>
-    <row r="40" spans="1:15">
+    <row r="40" spans="1:15" hidden="1">
       <c r="A40" s="44">
         <v>39</v>
       </c>
@@ -57063,7 +57064,7 @@
       <c r="N40" s="29"/>
       <c r="O40" s="53"/>
     </row>
-    <row r="41" spans="1:15">
+    <row r="41" spans="1:15" hidden="1">
       <c r="A41" s="44">
         <v>40</v>
       </c>
@@ -57101,7 +57102,7 @@
       <c r="N41" s="29"/>
       <c r="O41" s="53"/>
     </row>
-    <row r="42" spans="1:15">
+    <row r="42" spans="1:15" hidden="1">
       <c r="A42" s="44">
         <v>41</v>
       </c>
@@ -57139,7 +57140,7 @@
       <c r="N42" s="29"/>
       <c r="O42" s="53"/>
     </row>
-    <row r="43" spans="1:15">
+    <row r="43" spans="1:15" hidden="1">
       <c r="A43" s="44">
         <v>42</v>
       </c>
@@ -57225,7 +57226,7 @@
         <v>4900001801</v>
       </c>
     </row>
-    <row r="45" spans="1:15">
+    <row r="45" spans="1:15" hidden="1">
       <c r="A45" s="44">
         <v>44</v>
       </c>
@@ -57359,7 +57360,7 @@
         <v>4900001916</v>
       </c>
     </row>
-    <row r="48" spans="1:15">
+    <row r="48" spans="1:15" hidden="1">
       <c r="A48" s="44">
         <v>47</v>
       </c>
@@ -57397,7 +57398,7 @@
       <c r="N48" s="29"/>
       <c r="O48" s="53"/>
     </row>
-    <row r="49" spans="1:15">
+    <row r="49" spans="1:15" hidden="1">
       <c r="A49" s="44">
         <v>48</v>
       </c>
@@ -57435,7 +57436,7 @@
       <c r="N49" s="29"/>
       <c r="O49" s="53"/>
     </row>
-    <row r="50" spans="1:15">
+    <row r="50" spans="1:15" hidden="1">
       <c r="A50" s="44">
         <v>49</v>
       </c>
@@ -57521,7 +57522,7 @@
         <v>4900007935</v>
       </c>
     </row>
-    <row r="52" spans="1:15">
+    <row r="52" spans="1:15" hidden="1">
       <c r="A52" s="44">
         <v>51</v>
       </c>
@@ -57607,7 +57608,7 @@
         <v>4900003719</v>
       </c>
     </row>
-    <row r="54" spans="1:15">
+    <row r="54" spans="1:15" hidden="1">
       <c r="A54" s="44">
         <v>53</v>
       </c>
@@ -57645,7 +57646,7 @@
       <c r="N54" s="29"/>
       <c r="O54" s="53"/>
     </row>
-    <row r="55" spans="1:15">
+    <row r="55" spans="1:15" hidden="1">
       <c r="A55" s="44">
         <v>54</v>
       </c>
@@ -57683,7 +57684,7 @@
       <c r="N55" s="29"/>
       <c r="O55" s="53"/>
     </row>
-    <row r="56" spans="1:15">
+    <row r="56" spans="1:15" hidden="1">
       <c r="A56" s="44">
         <v>55</v>
       </c>
@@ -57769,7 +57770,7 @@
         <v>4900002656</v>
       </c>
     </row>
-    <row r="58" spans="1:15">
+    <row r="58" spans="1:15" hidden="1">
       <c r="A58" s="44">
         <v>57</v>
       </c>
@@ -57807,7 +57808,7 @@
       <c r="N58" s="29"/>
       <c r="O58" s="53"/>
     </row>
-    <row r="59" spans="1:15">
+    <row r="59" spans="1:15" hidden="1">
       <c r="A59" s="44">
         <v>58</v>
       </c>
@@ -57845,7 +57846,7 @@
       <c r="N59" s="29"/>
       <c r="O59" s="53"/>
     </row>
-    <row r="60" spans="1:15">
+    <row r="60" spans="1:15" hidden="1">
       <c r="A60" s="44">
         <v>59</v>
       </c>
@@ -57883,7 +57884,7 @@
       <c r="N60" s="29"/>
       <c r="O60" s="53"/>
     </row>
-    <row r="61" spans="1:15">
+    <row r="61" spans="1:15" hidden="1">
       <c r="A61" s="44">
         <v>60</v>
       </c>
@@ -57921,7 +57922,7 @@
       <c r="N61" s="29"/>
       <c r="O61" s="53"/>
     </row>
-    <row r="62" spans="1:15">
+    <row r="62" spans="1:15" hidden="1">
       <c r="A62" s="44">
         <v>61</v>
       </c>
@@ -58007,7 +58008,7 @@
         <v>2500005801</v>
       </c>
     </row>
-    <row r="64" spans="1:15">
+    <row r="64" spans="1:15" hidden="1">
       <c r="A64" s="44">
         <v>63</v>
       </c>
@@ -58045,7 +58046,7 @@
       <c r="N64" s="29"/>
       <c r="O64" s="53"/>
     </row>
-    <row r="65" spans="1:15">
+    <row r="65" spans="1:15" hidden="1">
       <c r="A65" s="44">
         <v>64</v>
       </c>
@@ -58083,7 +58084,7 @@
       <c r="N65" s="29"/>
       <c r="O65" s="53"/>
     </row>
-    <row r="66" spans="1:15">
+    <row r="66" spans="1:15" hidden="1">
       <c r="A66" s="44">
         <v>65</v>
       </c>
@@ -58121,7 +58122,7 @@
       <c r="N66" s="29"/>
       <c r="O66" s="53"/>
     </row>
-    <row r="67" spans="1:15">
+    <row r="67" spans="1:15" hidden="1">
       <c r="A67" s="44">
         <v>66</v>
       </c>
@@ -58159,7 +58160,7 @@
       <c r="N67" s="29"/>
       <c r="O67" s="53"/>
     </row>
-    <row r="68" spans="1:15">
+    <row r="68" spans="1:15" hidden="1">
       <c r="A68" s="44">
         <v>67</v>
       </c>
@@ -58197,7 +58198,7 @@
       <c r="N68" s="29"/>
       <c r="O68" s="53"/>
     </row>
-    <row r="69" spans="1:15">
+    <row r="69" spans="1:15" hidden="1">
       <c r="A69" s="44">
         <v>68</v>
       </c>
@@ -58235,7 +58236,7 @@
       <c r="N69" s="29"/>
       <c r="O69" s="53"/>
     </row>
-    <row r="70" spans="1:15">
+    <row r="70" spans="1:15" hidden="1">
       <c r="A70" s="44">
         <v>69</v>
       </c>
@@ -58273,7 +58274,7 @@
       <c r="N70" s="29"/>
       <c r="O70" s="53"/>
     </row>
-    <row r="71" spans="1:15">
+    <row r="71" spans="1:15" hidden="1">
       <c r="A71" s="44">
         <v>70</v>
       </c>
@@ -58311,7 +58312,7 @@
       <c r="N71" s="29"/>
       <c r="O71" s="53"/>
     </row>
-    <row r="72" spans="1:15">
+    <row r="72" spans="1:15" hidden="1">
       <c r="A72" s="44">
         <v>71</v>
       </c>
@@ -58349,7 +58350,7 @@
       <c r="N72" s="29"/>
       <c r="O72" s="53"/>
     </row>
-    <row r="73" spans="1:15">
+    <row r="73" spans="1:15" hidden="1">
       <c r="A73" s="44">
         <v>72</v>
       </c>
@@ -58387,7 +58388,7 @@
       <c r="N73" s="29"/>
       <c r="O73" s="53"/>
     </row>
-    <row r="74" spans="1:15">
+    <row r="74" spans="1:15" hidden="1">
       <c r="A74" s="44">
         <v>73</v>
       </c>
@@ -58473,7 +58474,7 @@
         <v>4900007938</v>
       </c>
     </row>
-    <row r="76" spans="1:15">
+    <row r="76" spans="1:15" hidden="1">
       <c r="A76" s="44">
         <v>75</v>
       </c>
@@ -58511,7 +58512,7 @@
       <c r="N76" s="29"/>
       <c r="O76" s="53"/>
     </row>
-    <row r="77" spans="1:15">
+    <row r="77" spans="1:15" hidden="1">
       <c r="A77" s="44">
         <v>76</v>
       </c>
@@ -58549,7 +58550,7 @@
       <c r="N77" s="29"/>
       <c r="O77" s="53"/>
     </row>
-    <row r="78" spans="1:15">
+    <row r="78" spans="1:15" hidden="1">
       <c r="A78" s="44">
         <v>77</v>
       </c>
@@ -58587,7 +58588,7 @@
       <c r="N78" s="29"/>
       <c r="O78" s="53"/>
     </row>
-    <row r="79" spans="1:15">
+    <row r="79" spans="1:15" hidden="1">
       <c r="A79" s="44">
         <v>78</v>
       </c>
@@ -58673,7 +58674,7 @@
         <v>8616200297</v>
       </c>
     </row>
-    <row r="81" spans="1:15">
+    <row r="81" spans="1:15" hidden="1">
       <c r="A81" s="44">
         <v>80</v>
       </c>
@@ -58759,7 +58760,7 @@
         <v>4900004754</v>
       </c>
     </row>
-    <row r="83" spans="1:15">
+    <row r="83" spans="1:15" hidden="1">
       <c r="A83" s="44">
         <v>82</v>
       </c>
@@ -58797,7 +58798,7 @@
       <c r="N83" s="29"/>
       <c r="O83" s="53"/>
     </row>
-    <row r="84" spans="1:15">
+    <row r="84" spans="1:15" hidden="1">
       <c r="A84" s="44">
         <v>83</v>
       </c>
@@ -58835,7 +58836,7 @@
       <c r="N84" s="29"/>
       <c r="O84" s="53"/>
     </row>
-    <row r="85" spans="1:15">
+    <row r="85" spans="1:15" hidden="1">
       <c r="A85" s="44">
         <v>84</v>
       </c>
@@ -58873,7 +58874,7 @@
       <c r="N85" s="29"/>
       <c r="O85" s="53"/>
     </row>
-    <row r="86" spans="1:15">
+    <row r="86" spans="1:15" hidden="1">
       <c r="A86" s="44">
         <v>85</v>
       </c>
@@ -58911,7 +58912,7 @@
       <c r="N86" s="29"/>
       <c r="O86" s="53"/>
     </row>
-    <row r="87" spans="1:15">
+    <row r="87" spans="1:15" hidden="1">
       <c r="A87" s="44">
         <v>86</v>
       </c>
@@ -58949,7 +58950,7 @@
       <c r="N87" s="29"/>
       <c r="O87" s="53"/>
     </row>
-    <row r="88" spans="1:15">
+    <row r="88" spans="1:15" hidden="1">
       <c r="A88" s="44">
         <v>87</v>
       </c>
@@ -58987,7 +58988,7 @@
       <c r="N88" s="29"/>
       <c r="O88" s="53"/>
     </row>
-    <row r="89" spans="1:15">
+    <row r="89" spans="1:15" hidden="1">
       <c r="A89" s="44">
         <v>88</v>
       </c>
@@ -59025,7 +59026,7 @@
       <c r="N89" s="29"/>
       <c r="O89" s="53"/>
     </row>
-    <row r="90" spans="1:15">
+    <row r="90" spans="1:15" hidden="1">
       <c r="A90" s="44">
         <v>89</v>
       </c>
@@ -59063,7 +59064,7 @@
       <c r="N90" s="29"/>
       <c r="O90" s="53"/>
     </row>
-    <row r="91" spans="1:15">
+    <row r="91" spans="1:15" hidden="1">
       <c r="A91" s="44">
         <v>90</v>
       </c>
@@ -59101,7 +59102,7 @@
       <c r="N91" s="29"/>
       <c r="O91" s="53"/>
     </row>
-    <row r="92" spans="1:15">
+    <row r="92" spans="1:15" hidden="1">
       <c r="A92" s="44">
         <v>91</v>
       </c>
@@ -59139,7 +59140,7 @@
       <c r="N92" s="29"/>
       <c r="O92" s="53"/>
     </row>
-    <row r="93" spans="1:15">
+    <row r="93" spans="1:15" hidden="1">
       <c r="A93" s="44">
         <v>92</v>
       </c>
@@ -59177,7 +59178,7 @@
       <c r="N93" s="29"/>
       <c r="O93" s="53"/>
     </row>
-    <row r="94" spans="1:15">
+    <row r="94" spans="1:15" hidden="1">
       <c r="A94" s="44">
         <v>93</v>
       </c>
@@ -59311,7 +59312,7 @@
         <v>2500005802</v>
       </c>
     </row>
-    <row r="97" spans="1:15">
+    <row r="97" spans="1:15" hidden="1">
       <c r="A97" s="44">
         <v>96</v>
       </c>
@@ -59349,7 +59350,7 @@
       <c r="N97" s="29"/>
       <c r="O97" s="53"/>
     </row>
-    <row r="98" spans="1:15">
+    <row r="98" spans="1:15" hidden="1">
       <c r="A98" s="44">
         <v>97</v>
       </c>
@@ -59387,7 +59388,7 @@
       <c r="N98" s="29"/>
       <c r="O98" s="53"/>
     </row>
-    <row r="99" spans="1:15">
+    <row r="99" spans="1:15" hidden="1">
       <c r="A99" s="44">
         <v>98</v>
       </c>
@@ -59425,7 +59426,7 @@
       <c r="N99" s="29"/>
       <c r="O99" s="53"/>
     </row>
-    <row r="100" spans="1:15">
+    <row r="100" spans="1:15" hidden="1">
       <c r="A100" s="44">
         <v>99</v>
       </c>
@@ -59463,7 +59464,7 @@
       <c r="N100" s="29"/>
       <c r="O100" s="53"/>
     </row>
-    <row r="101" spans="1:15">
+    <row r="101" spans="1:15" hidden="1">
       <c r="A101" s="44">
         <v>100</v>
       </c>
@@ -59501,7 +59502,7 @@
       <c r="N101" s="29"/>
       <c r="O101" s="53"/>
     </row>
-    <row r="102" spans="1:15">
+    <row r="102" spans="1:15" hidden="1">
       <c r="A102" s="44">
         <v>101</v>
       </c>
@@ -59539,7 +59540,7 @@
       <c r="N102" s="29"/>
       <c r="O102" s="53"/>
     </row>
-    <row r="103" spans="1:15">
+    <row r="103" spans="1:15" hidden="1">
       <c r="A103" s="44">
         <v>102</v>
       </c>
@@ -59577,7 +59578,7 @@
       <c r="N103" s="29"/>
       <c r="O103" s="53"/>
     </row>
-    <row r="104" spans="1:15">
+    <row r="104" spans="1:15" hidden="1">
       <c r="A104" s="44">
         <v>103</v>
       </c>
@@ -59615,7 +59616,7 @@
       <c r="N104" s="29"/>
       <c r="O104" s="53"/>
     </row>
-    <row r="105" spans="1:15">
+    <row r="105" spans="1:15" hidden="1">
       <c r="A105" s="44">
         <v>104</v>
       </c>
@@ -59653,7 +59654,7 @@
       <c r="N105" s="29"/>
       <c r="O105" s="53"/>
     </row>
-    <row r="106" spans="1:15">
+    <row r="106" spans="1:15" hidden="1">
       <c r="A106" s="44">
         <v>105</v>
       </c>
@@ -59691,7 +59692,7 @@
       <c r="N106" s="29"/>
       <c r="O106" s="53"/>
     </row>
-    <row r="107" spans="1:15">
+    <row r="107" spans="1:15" hidden="1">
       <c r="A107" s="44">
         <v>106</v>
       </c>
@@ -59729,7 +59730,7 @@
       <c r="N107" s="29"/>
       <c r="O107" s="53"/>
     </row>
-    <row r="108" spans="1:15">
+    <row r="108" spans="1:15" hidden="1">
       <c r="A108" s="44">
         <v>107</v>
       </c>
@@ -59767,7 +59768,7 @@
       <c r="N108" s="29"/>
       <c r="O108" s="53"/>
     </row>
-    <row r="109" spans="1:15">
+    <row r="109" spans="1:15" hidden="1">
       <c r="A109" s="44">
         <v>108</v>
       </c>
@@ -59805,7 +59806,7 @@
       <c r="N109" s="29"/>
       <c r="O109" s="53"/>
     </row>
-    <row r="110" spans="1:15">
+    <row r="110" spans="1:15" hidden="1">
       <c r="A110" s="44">
         <v>109</v>
       </c>
@@ -59843,7 +59844,7 @@
       <c r="N110" s="29"/>
       <c r="O110" s="53"/>
     </row>
-    <row r="111" spans="1:15">
+    <row r="111" spans="1:15" hidden="1">
       <c r="A111" s="44">
         <v>110</v>
       </c>
@@ -59881,7 +59882,7 @@
       <c r="N111" s="29"/>
       <c r="O111" s="53"/>
     </row>
-    <row r="112" spans="1:15">
+    <row r="112" spans="1:15" hidden="1">
       <c r="A112" s="44">
         <v>111</v>
       </c>
@@ -59919,7 +59920,7 @@
       <c r="N112" s="29"/>
       <c r="O112" s="53"/>
     </row>
-    <row r="113" spans="1:15">
+    <row r="113" spans="1:15" hidden="1">
       <c r="A113" s="44">
         <v>112</v>
       </c>
@@ -59957,7 +59958,7 @@
       <c r="N113" s="29"/>
       <c r="O113" s="53"/>
     </row>
-    <row r="114" spans="1:15">
+    <row r="114" spans="1:15" hidden="1">
       <c r="A114" s="44">
         <v>113</v>
       </c>
@@ -59995,7 +59996,7 @@
       <c r="N114" s="29"/>
       <c r="O114" s="53"/>
     </row>
-    <row r="115" spans="1:15">
+    <row r="115" spans="1:15" hidden="1">
       <c r="A115" s="44">
         <v>114</v>
       </c>
@@ -60033,7 +60034,7 @@
       <c r="N115" s="29"/>
       <c r="O115" s="53"/>
     </row>
-    <row r="116" spans="1:15">
+    <row r="116" spans="1:15" hidden="1">
       <c r="A116" s="44">
         <v>115</v>
       </c>
@@ -60119,7 +60120,7 @@
         <v>2500006153</v>
       </c>
     </row>
-    <row r="118" spans="1:15">
+    <row r="118" spans="1:15" hidden="1">
       <c r="A118" s="44">
         <v>117</v>
       </c>
@@ -60157,7 +60158,7 @@
       <c r="N118" s="29"/>
       <c r="O118" s="53"/>
     </row>
-    <row r="119" spans="1:15">
+    <row r="119" spans="1:15" hidden="1">
       <c r="A119" s="44">
         <v>118</v>
       </c>
@@ -60195,7 +60196,7 @@
       <c r="N119" s="29"/>
       <c r="O119" s="53"/>
     </row>
-    <row r="120" spans="1:15">
+    <row r="120" spans="1:15" hidden="1">
       <c r="A120" s="44">
         <v>119</v>
       </c>
@@ -60233,7 +60234,7 @@
       <c r="N120" s="29"/>
       <c r="O120" s="53"/>
     </row>
-    <row r="121" spans="1:15">
+    <row r="121" spans="1:15" hidden="1">
       <c r="A121" s="44">
         <v>120</v>
       </c>
@@ -60271,7 +60272,7 @@
       <c r="N121" s="29"/>
       <c r="O121" s="53"/>
     </row>
-    <row r="122" spans="1:15">
+    <row r="122" spans="1:15" hidden="1">
       <c r="A122" s="44">
         <v>121</v>
       </c>
@@ -60309,7 +60310,7 @@
       <c r="N122" s="29"/>
       <c r="O122" s="53"/>
     </row>
-    <row r="123" spans="1:15">
+    <row r="123" spans="1:15" hidden="1">
       <c r="A123" s="44">
         <v>122</v>
       </c>
@@ -60347,7 +60348,7 @@
       <c r="N123" s="29"/>
       <c r="O123" s="53"/>
     </row>
-    <row r="124" spans="1:15">
+    <row r="124" spans="1:15" hidden="1">
       <c r="A124" s="44">
         <v>123</v>
       </c>
@@ -60385,7 +60386,7 @@
       <c r="N124" s="29"/>
       <c r="O124" s="53"/>
     </row>
-    <row r="125" spans="1:15">
+    <row r="125" spans="1:15" hidden="1">
       <c r="A125" s="44">
         <v>124</v>
       </c>
@@ -60423,7 +60424,7 @@
       <c r="N125" s="29"/>
       <c r="O125" s="53"/>
     </row>
-    <row r="126" spans="1:15">
+    <row r="126" spans="1:15" hidden="1">
       <c r="A126" s="44">
         <v>125</v>
       </c>
@@ -60461,7 +60462,7 @@
       <c r="N126" s="29"/>
       <c r="O126" s="53"/>
     </row>
-    <row r="127" spans="1:15">
+    <row r="127" spans="1:15" hidden="1">
       <c r="A127" s="44">
         <v>126</v>
       </c>
@@ -60547,7 +60548,7 @@
         <v>8616200296</v>
       </c>
     </row>
-    <row r="129" spans="1:15">
+    <row r="129" spans="1:15" hidden="1">
       <c r="A129" s="44">
         <v>128</v>
       </c>
@@ -60585,7 +60586,7 @@
       <c r="N129" s="29"/>
       <c r="O129" s="53"/>
     </row>
-    <row r="130" spans="1:15">
+    <row r="130" spans="1:15" hidden="1">
       <c r="A130" s="44">
         <v>129</v>
       </c>
@@ -60623,7 +60624,7 @@
       <c r="N130" s="29"/>
       <c r="O130" s="53"/>
     </row>
-    <row r="131" spans="1:15">
+    <row r="131" spans="1:15" hidden="1">
       <c r="A131" s="44">
         <v>130</v>
       </c>
@@ -60661,7 +60662,7 @@
       <c r="N131" s="29"/>
       <c r="O131" s="53"/>
     </row>
-    <row r="132" spans="1:15">
+    <row r="132" spans="1:15" hidden="1">
       <c r="A132" s="44">
         <v>131</v>
       </c>
@@ -60699,7 +60700,7 @@
       <c r="N132" s="29"/>
       <c r="O132" s="53"/>
     </row>
-    <row r="133" spans="1:15">
+    <row r="133" spans="1:15" hidden="1">
       <c r="A133" s="44">
         <v>132</v>
       </c>
@@ -60737,7 +60738,7 @@
       <c r="N133" s="29"/>
       <c r="O133" s="53"/>
     </row>
-    <row r="134" spans="1:15">
+    <row r="134" spans="1:15" hidden="1">
       <c r="A134" s="44">
         <v>133</v>
       </c>
@@ -60775,7 +60776,7 @@
       <c r="N134" s="29"/>
       <c r="O134" s="53"/>
     </row>
-    <row r="135" spans="1:15">
+    <row r="135" spans="1:15" hidden="1">
       <c r="A135" s="44">
         <v>134</v>
       </c>
@@ -60813,7 +60814,7 @@
       <c r="N135" s="29"/>
       <c r="O135" s="53"/>
     </row>
-    <row r="136" spans="1:15">
+    <row r="136" spans="1:15" hidden="1">
       <c r="A136" s="44">
         <v>135</v>
       </c>
@@ -60851,7 +60852,7 @@
       <c r="N136" s="29"/>
       <c r="O136" s="53"/>
     </row>
-    <row r="137" spans="1:15">
+    <row r="137" spans="1:15" hidden="1">
       <c r="A137" s="44">
         <v>136</v>
       </c>
@@ -60937,7 +60938,7 @@
         <v>2500006151</v>
       </c>
     </row>
-    <row r="139" spans="1:15">
+    <row r="139" spans="1:15" hidden="1">
       <c r="A139" s="44">
         <v>138</v>
       </c>
@@ -60975,7 +60976,7 @@
       <c r="N139" s="29"/>
       <c r="O139" s="53"/>
     </row>
-    <row r="140" spans="1:15">
+    <row r="140" spans="1:15" hidden="1">
       <c r="A140" s="44">
         <v>139</v>
       </c>
@@ -61013,7 +61014,7 @@
       <c r="N140" s="29"/>
       <c r="O140" s="53"/>
     </row>
-    <row r="141" spans="1:15">
+    <row r="141" spans="1:15" hidden="1">
       <c r="A141" s="44">
         <v>140</v>
       </c>
@@ -61051,7 +61052,7 @@
       <c r="N141" s="29"/>
       <c r="O141" s="53"/>
     </row>
-    <row r="142" spans="1:15">
+    <row r="142" spans="1:15" hidden="1">
       <c r="A142" s="44">
         <v>141</v>
       </c>
@@ -61089,7 +61090,7 @@
       <c r="N142" s="29"/>
       <c r="O142" s="53"/>
     </row>
-    <row r="143" spans="1:15">
+    <row r="143" spans="1:15" hidden="1">
       <c r="A143" s="44">
         <v>142</v>
       </c>
@@ -61127,7 +61128,7 @@
       <c r="N143" s="29"/>
       <c r="O143" s="53"/>
     </row>
-    <row r="144" spans="1:15">
+    <row r="144" spans="1:15" hidden="1">
       <c r="A144" s="44">
         <v>143</v>
       </c>
@@ -61165,7 +61166,7 @@
       <c r="N144" s="29"/>
       <c r="O144" s="53"/>
     </row>
-    <row r="145" spans="1:15">
+    <row r="145" spans="1:15" hidden="1">
       <c r="A145" s="44">
         <v>144</v>
       </c>
@@ -61203,7 +61204,7 @@
       <c r="N145" s="29"/>
       <c r="O145" s="53"/>
     </row>
-    <row r="146" spans="1:15">
+    <row r="146" spans="1:15" hidden="1">
       <c r="A146" s="44">
         <v>145</v>
       </c>
@@ -61241,7 +61242,7 @@
       <c r="N146" s="29"/>
       <c r="O146" s="53"/>
     </row>
-    <row r="147" spans="1:15">
+    <row r="147" spans="1:15" hidden="1">
       <c r="A147" s="44">
         <v>146</v>
       </c>
@@ -61279,7 +61280,7 @@
       <c r="N147" s="29"/>
       <c r="O147" s="53"/>
     </row>
-    <row r="148" spans="1:15">
+    <row r="148" spans="1:15" hidden="1">
       <c r="A148" s="44">
         <v>147</v>
       </c>
@@ -61317,7 +61318,7 @@
       <c r="N148" s="29"/>
       <c r="O148" s="53"/>
     </row>
-    <row r="149" spans="1:15">
+    <row r="149" spans="1:15" hidden="1">
       <c r="A149" s="44">
         <v>148</v>
       </c>
@@ -61355,7 +61356,7 @@
       <c r="N149" s="29"/>
       <c r="O149" s="53"/>
     </row>
-    <row r="150" spans="1:15">
+    <row r="150" spans="1:15" hidden="1">
       <c r="A150" s="44">
         <v>149</v>
       </c>
@@ -61393,7 +61394,7 @@
       <c r="N150" s="29"/>
       <c r="O150" s="53"/>
     </row>
-    <row r="151" spans="1:15">
+    <row r="151" spans="1:15" hidden="1">
       <c r="A151" s="44">
         <v>150</v>
       </c>
@@ -61431,7 +61432,7 @@
       <c r="N151" s="29"/>
       <c r="O151" s="53"/>
     </row>
-    <row r="152" spans="1:15">
+    <row r="152" spans="1:15" hidden="1">
       <c r="A152" s="44">
         <v>151</v>
       </c>
@@ -61469,7 +61470,7 @@
       <c r="N152" s="29"/>
       <c r="O152" s="53"/>
     </row>
-    <row r="153" spans="1:15">
+    <row r="153" spans="1:15" hidden="1">
       <c r="A153" s="44">
         <v>152</v>
       </c>
@@ -61507,7 +61508,7 @@
       <c r="N153" s="29"/>
       <c r="O153" s="53"/>
     </row>
-    <row r="154" spans="1:15">
+    <row r="154" spans="1:15" hidden="1">
       <c r="A154" s="44">
         <v>153</v>
       </c>
@@ -61545,7 +61546,7 @@
       <c r="N154" s="29"/>
       <c r="O154" s="53"/>
     </row>
-    <row r="155" spans="1:15">
+    <row r="155" spans="1:15" hidden="1">
       <c r="A155" s="44">
         <v>154</v>
       </c>
@@ -61583,7 +61584,7 @@
       <c r="N155" s="29"/>
       <c r="O155" s="53"/>
     </row>
-    <row r="156" spans="1:15">
+    <row r="156" spans="1:15" hidden="1">
       <c r="A156" s="44">
         <v>155</v>
       </c>
@@ -61621,7 +61622,7 @@
       <c r="N156" s="29"/>
       <c r="O156" s="53"/>
     </row>
-    <row r="157" spans="1:15">
+    <row r="157" spans="1:15" hidden="1">
       <c r="A157" s="44">
         <v>156</v>
       </c>
@@ -61659,7 +61660,7 @@
       <c r="N157" s="29"/>
       <c r="O157" s="53"/>
     </row>
-    <row r="158" spans="1:15">
+    <row r="158" spans="1:15" hidden="1">
       <c r="A158" s="44">
         <v>157</v>
       </c>
@@ -61697,7 +61698,7 @@
       <c r="N158" s="29"/>
       <c r="O158" s="53"/>
     </row>
-    <row r="159" spans="1:15">
+    <row r="159" spans="1:15" hidden="1">
       <c r="A159" s="44">
         <v>158</v>
       </c>
@@ -61735,7 +61736,7 @@
       <c r="N159" s="29"/>
       <c r="O159" s="53"/>
     </row>
-    <row r="160" spans="1:15">
+    <row r="160" spans="1:15" hidden="1">
       <c r="A160" s="44">
         <v>159</v>
       </c>
@@ -61773,7 +61774,7 @@
       <c r="N160" s="29"/>
       <c r="O160" s="53"/>
     </row>
-    <row r="161" spans="1:15">
+    <row r="161" spans="1:15" hidden="1">
       <c r="A161" s="44">
         <v>160</v>
       </c>
@@ -61811,7 +61812,7 @@
       <c r="N161" s="29"/>
       <c r="O161" s="53"/>
     </row>
-    <row r="162" spans="1:15">
+    <row r="162" spans="1:15" hidden="1">
       <c r="A162" s="44">
         <v>161</v>
       </c>
@@ -61849,7 +61850,7 @@
       <c r="N162" s="29"/>
       <c r="O162" s="53"/>
     </row>
-    <row r="163" spans="1:15">
+    <row r="163" spans="1:15" hidden="1">
       <c r="A163" s="44">
         <v>162</v>
       </c>
@@ -61935,7 +61936,7 @@
         <v>4900056109</v>
       </c>
     </row>
-    <row r="165" spans="1:15">
+    <row r="165" spans="1:15" hidden="1">
       <c r="A165" s="44">
         <v>164</v>
       </c>
@@ -61973,7 +61974,7 @@
       <c r="N165" s="29"/>
       <c r="O165" s="53"/>
     </row>
-    <row r="166" spans="1:15">
+    <row r="166" spans="1:15" hidden="1">
       <c r="A166" s="44">
         <v>165</v>
       </c>
@@ -62011,7 +62012,7 @@
       <c r="N166" s="29"/>
       <c r="O166" s="53"/>
     </row>
-    <row r="167" spans="1:15">
+    <row r="167" spans="1:15" hidden="1">
       <c r="A167" s="44">
         <v>166</v>
       </c>
@@ -62049,7 +62050,7 @@
       <c r="N167" s="29"/>
       <c r="O167" s="53"/>
     </row>
-    <row r="168" spans="1:15">
+    <row r="168" spans="1:15" hidden="1">
       <c r="A168" s="44">
         <v>167</v>
       </c>
@@ -62087,7 +62088,7 @@
       <c r="N168" s="29"/>
       <c r="O168" s="53"/>
     </row>
-    <row r="169" spans="1:15">
+    <row r="169" spans="1:15" hidden="1">
       <c r="A169" s="44">
         <v>168</v>
       </c>
@@ -62125,7 +62126,7 @@
       <c r="N169" s="29"/>
       <c r="O169" s="53"/>
     </row>
-    <row r="170" spans="1:15">
+    <row r="170" spans="1:15" hidden="1">
       <c r="A170" s="44">
         <v>169</v>
       </c>
@@ -62163,7 +62164,7 @@
       <c r="N170" s="29"/>
       <c r="O170" s="53"/>
     </row>
-    <row r="171" spans="1:15">
+    <row r="171" spans="1:15" hidden="1">
       <c r="A171" s="44">
         <v>170</v>
       </c>
@@ -62201,7 +62202,7 @@
       <c r="N171" s="29"/>
       <c r="O171" s="53"/>
     </row>
-    <row r="172" spans="1:15">
+    <row r="172" spans="1:15" hidden="1">
       <c r="A172" s="44">
         <v>171</v>
       </c>
@@ -62239,7 +62240,7 @@
       <c r="N172" s="29"/>
       <c r="O172" s="53"/>
     </row>
-    <row r="173" spans="1:15">
+    <row r="173" spans="1:15" hidden="1">
       <c r="A173" s="44">
         <v>172</v>
       </c>
@@ -62325,7 +62326,7 @@
         <v>4900056169</v>
       </c>
     </row>
-    <row r="175" spans="1:15">
+    <row r="175" spans="1:15" hidden="1">
       <c r="A175" s="44">
         <v>174</v>
       </c>
@@ -62363,7 +62364,7 @@
       <c r="N175" s="29"/>
       <c r="O175" s="53"/>
     </row>
-    <row r="176" spans="1:15">
+    <row r="176" spans="1:15" hidden="1">
       <c r="A176" s="44">
         <v>175</v>
       </c>
@@ -62401,7 +62402,7 @@
       <c r="N176" s="29"/>
       <c r="O176" s="53"/>
     </row>
-    <row r="177" spans="1:15">
+    <row r="177" spans="1:15" hidden="1">
       <c r="A177" s="44">
         <v>176</v>
       </c>
@@ -62439,7 +62440,7 @@
       <c r="N177" s="29"/>
       <c r="O177" s="53"/>
     </row>
-    <row r="178" spans="1:15">
+    <row r="178" spans="1:15" hidden="1">
       <c r="A178" s="44">
         <v>177</v>
       </c>
@@ -62477,7 +62478,7 @@
       <c r="N178" s="29"/>
       <c r="O178" s="53"/>
     </row>
-    <row r="179" spans="1:15">
+    <row r="179" spans="1:15" hidden="1">
       <c r="A179" s="44">
         <v>178</v>
       </c>
@@ -62515,7 +62516,7 @@
       <c r="N179" s="29"/>
       <c r="O179" s="53"/>
     </row>
-    <row r="180" spans="1:15">
+    <row r="180" spans="1:15" hidden="1">
       <c r="A180" s="44">
         <v>179</v>
       </c>
@@ -62553,7 +62554,7 @@
       <c r="N180" s="29"/>
       <c r="O180" s="53"/>
     </row>
-    <row r="181" spans="1:15">
+    <row r="181" spans="1:15" hidden="1">
       <c r="A181" s="44">
         <v>180</v>
       </c>
@@ -62591,7 +62592,7 @@
       <c r="N181" s="29"/>
       <c r="O181" s="53"/>
     </row>
-    <row r="182" spans="1:15">
+    <row r="182" spans="1:15" hidden="1">
       <c r="A182" s="44">
         <v>181</v>
       </c>
@@ -62629,7 +62630,7 @@
       <c r="N182" s="29"/>
       <c r="O182" s="53"/>
     </row>
-    <row r="183" spans="1:15">
+    <row r="183" spans="1:15" hidden="1">
       <c r="A183" s="44">
         <v>182</v>
       </c>
@@ -62667,7 +62668,7 @@
       <c r="N183" s="29"/>
       <c r="O183" s="53"/>
     </row>
-    <row r="184" spans="1:15">
+    <row r="184" spans="1:15" hidden="1">
       <c r="A184" s="44">
         <v>183</v>
       </c>
@@ -62705,7 +62706,7 @@
       <c r="N184" s="29"/>
       <c r="O184" s="53"/>
     </row>
-    <row r="185" spans="1:15">
+    <row r="185" spans="1:15" hidden="1">
       <c r="A185" s="44">
         <v>184</v>
       </c>
@@ -62743,7 +62744,7 @@
       <c r="N185" s="29"/>
       <c r="O185" s="53"/>
     </row>
-    <row r="186" spans="1:15">
+    <row r="186" spans="1:15" hidden="1">
       <c r="A186" s="44">
         <v>185</v>
       </c>
@@ -62829,7 +62830,7 @@
         <v>5817600231</v>
       </c>
     </row>
-    <row r="188" spans="1:15">
+    <row r="188" spans="1:15" hidden="1">
       <c r="A188" s="44">
         <v>187</v>
       </c>
@@ -62867,7 +62868,7 @@
       <c r="N188" s="29"/>
       <c r="O188" s="53"/>
     </row>
-    <row r="189" spans="1:15">
+    <row r="189" spans="1:15" hidden="1">
       <c r="A189" s="44">
         <v>188</v>
       </c>
@@ -62905,7 +62906,7 @@
       <c r="N189" s="29"/>
       <c r="O189" s="53"/>
     </row>
-    <row r="190" spans="1:15">
+    <row r="190" spans="1:15" hidden="1">
       <c r="A190" s="44">
         <v>189</v>
       </c>
@@ -62991,7 +62992,7 @@
         <v>5817600230</v>
       </c>
     </row>
-    <row r="192" spans="1:15">
+    <row r="192" spans="1:15" hidden="1">
       <c r="A192" s="44">
         <v>191</v>
       </c>
@@ -63029,7 +63030,7 @@
       <c r="N192" s="29"/>
       <c r="O192" s="53"/>
     </row>
-    <row r="193" spans="1:15">
+    <row r="193" spans="1:15" hidden="1">
       <c r="A193" s="44">
         <v>192</v>
       </c>
@@ -63067,7 +63068,7 @@
       <c r="N193" s="29"/>
       <c r="O193" s="53"/>
     </row>
-    <row r="194" spans="1:15">
+    <row r="194" spans="1:15" hidden="1">
       <c r="A194" s="44">
         <v>193</v>
       </c>
@@ -63105,7 +63106,7 @@
       <c r="N194" s="29"/>
       <c r="O194" s="53"/>
     </row>
-    <row r="195" spans="1:15">
+    <row r="195" spans="1:15" hidden="1">
       <c r="A195" s="44">
         <v>194</v>
       </c>
@@ -63143,7 +63144,7 @@
       <c r="N195" s="29"/>
       <c r="O195" s="53"/>
     </row>
-    <row r="196" spans="1:15">
+    <row r="196" spans="1:15" hidden="1">
       <c r="A196" s="44">
         <v>195</v>
       </c>
@@ -63181,7 +63182,7 @@
       <c r="N196" s="29"/>
       <c r="O196" s="53"/>
     </row>
-    <row r="197" spans="1:15">
+    <row r="197" spans="1:15" hidden="1">
       <c r="A197" s="44">
         <v>196</v>
       </c>
@@ -63219,7 +63220,7 @@
       <c r="N197" s="29"/>
       <c r="O197" s="53"/>
     </row>
-    <row r="198" spans="1:15">
+    <row r="198" spans="1:15" hidden="1">
       <c r="A198" s="44">
         <v>197</v>
       </c>
@@ -63257,7 +63258,7 @@
       <c r="N198" s="29"/>
       <c r="O198" s="53"/>
     </row>
-    <row r="199" spans="1:15">
+    <row r="199" spans="1:15" hidden="1">
       <c r="A199" s="44">
         <v>198</v>
       </c>
@@ -63295,7 +63296,7 @@
       <c r="N199" s="29"/>
       <c r="O199" s="53"/>
     </row>
-    <row r="200" spans="1:15">
+    <row r="200" spans="1:15" hidden="1">
       <c r="A200" s="44">
         <v>199</v>
       </c>
@@ -63333,7 +63334,7 @@
       <c r="N200" s="29"/>
       <c r="O200" s="53"/>
     </row>
-    <row r="201" spans="1:15">
+    <row r="201" spans="1:15" hidden="1">
       <c r="A201" s="44">
         <v>200</v>
       </c>
@@ -63371,7 +63372,7 @@
       <c r="N201" s="29"/>
       <c r="O201" s="53"/>
     </row>
-    <row r="202" spans="1:15">
+    <row r="202" spans="1:15" hidden="1">
       <c r="A202" s="44">
         <v>201</v>
       </c>
@@ -63457,7 +63458,7 @@
         <v>4900001806</v>
       </c>
     </row>
-    <row r="204" spans="1:15">
+    <row r="204" spans="1:15" hidden="1">
       <c r="A204" s="44">
         <v>203</v>
       </c>
@@ -63495,7 +63496,7 @@
       <c r="N204" s="29"/>
       <c r="O204" s="53"/>
     </row>
-    <row r="205" spans="1:15">
+    <row r="205" spans="1:15" hidden="1">
       <c r="A205" s="44">
         <v>204</v>
       </c>
@@ -63533,7 +63534,7 @@
       <c r="N205" s="29"/>
       <c r="O205" s="53"/>
     </row>
-    <row r="206" spans="1:15">
+    <row r="206" spans="1:15" hidden="1">
       <c r="A206" s="44">
         <v>205</v>
       </c>
@@ -63571,7 +63572,7 @@
       <c r="N206" s="29"/>
       <c r="O206" s="53"/>
     </row>
-    <row r="207" spans="1:15">
+    <row r="207" spans="1:15" hidden="1">
       <c r="A207" s="44">
         <v>206</v>
       </c>
@@ -63609,7 +63610,7 @@
       <c r="N207" s="29"/>
       <c r="O207" s="53"/>
     </row>
-    <row r="208" spans="1:15">
+    <row r="208" spans="1:15" hidden="1">
       <c r="A208" s="44">
         <v>207</v>
       </c>
@@ -63647,7 +63648,7 @@
       <c r="N208" s="29"/>
       <c r="O208" s="53"/>
     </row>
-    <row r="209" spans="1:15">
+    <row r="209" spans="1:15" hidden="1">
       <c r="A209" s="44">
         <v>208</v>
       </c>
@@ -63685,7 +63686,7 @@
       <c r="N209" s="29"/>
       <c r="O209" s="53"/>
     </row>
-    <row r="210" spans="1:15">
+    <row r="210" spans="1:15" hidden="1">
       <c r="A210" s="44">
         <v>209</v>
       </c>
@@ -63723,7 +63724,7 @@
       <c r="N210" s="29"/>
       <c r="O210" s="53"/>
     </row>
-    <row r="211" spans="1:15">
+    <row r="211" spans="1:15" hidden="1">
       <c r="A211" s="44">
         <v>210</v>
       </c>
@@ -63761,7 +63762,7 @@
       <c r="N211" s="29"/>
       <c r="O211" s="53"/>
     </row>
-    <row r="212" spans="1:15">
+    <row r="212" spans="1:15" hidden="1">
       <c r="A212" s="44">
         <v>211</v>
       </c>
@@ -63847,7 +63848,7 @@
         <v>8390000597</v>
       </c>
     </row>
-    <row r="214" spans="1:15">
+    <row r="214" spans="1:15" hidden="1">
       <c r="A214" s="44">
         <v>213</v>
       </c>
@@ -63885,7 +63886,7 @@
       <c r="N214" s="29"/>
       <c r="O214" s="53"/>
     </row>
-    <row r="215" spans="1:15">
+    <row r="215" spans="1:15" hidden="1">
       <c r="A215" s="44">
         <v>214</v>
       </c>
@@ -63923,7 +63924,7 @@
       <c r="N215" s="29"/>
       <c r="O215" s="53"/>
     </row>
-    <row r="216" spans="1:15">
+    <row r="216" spans="1:15" hidden="1">
       <c r="A216" s="44">
         <v>215</v>
       </c>
@@ -63961,7 +63962,7 @@
       <c r="N216" s="29"/>
       <c r="O216" s="53"/>
     </row>
-    <row r="217" spans="1:15">
+    <row r="217" spans="1:15" hidden="1">
       <c r="A217" s="44">
         <v>216</v>
       </c>
@@ -63999,7 +64000,7 @@
       <c r="N217" s="29"/>
       <c r="O217" s="53"/>
     </row>
-    <row r="218" spans="1:15">
+    <row r="218" spans="1:15" hidden="1">
       <c r="A218" s="44">
         <v>217</v>
       </c>
@@ -64085,7 +64086,7 @@
         <v>4900055769</v>
       </c>
     </row>
-    <row r="220" spans="1:15">
+    <row r="220" spans="1:15" hidden="1">
       <c r="A220" s="44">
         <v>219</v>
       </c>
@@ -64123,7 +64124,7 @@
       <c r="N220" s="29"/>
       <c r="O220" s="53"/>
     </row>
-    <row r="221" spans="1:15">
+    <row r="221" spans="1:15" hidden="1">
       <c r="A221" s="44">
         <v>220</v>
       </c>
@@ -64209,7 +64210,7 @@
         <v>8390000575</v>
       </c>
     </row>
-    <row r="223" spans="1:15">
+    <row r="223" spans="1:15" hidden="1">
       <c r="A223" s="44">
         <v>222</v>
       </c>
@@ -64247,7 +64248,7 @@
       <c r="N223" s="29"/>
       <c r="O223" s="53"/>
     </row>
-    <row r="224" spans="1:15">
+    <row r="224" spans="1:15" hidden="1">
       <c r="A224" s="44">
         <v>223</v>
       </c>
@@ -64333,7 +64334,7 @@
         <v>4900055771</v>
       </c>
     </row>
-    <row r="226" spans="1:15">
+    <row r="226" spans="1:15" hidden="1">
       <c r="A226" s="44">
         <v>225</v>
       </c>
@@ -64419,7 +64420,7 @@
         <v>4900055773</v>
       </c>
     </row>
-    <row r="228" spans="1:15">
+    <row r="228" spans="1:15" hidden="1">
       <c r="A228" s="44">
         <v>227</v>
       </c>
@@ -64457,7 +64458,7 @@
       <c r="N228" s="29"/>
       <c r="O228" s="48"/>
     </row>
-    <row r="229" spans="1:15">
+    <row r="229" spans="1:15" hidden="1">
       <c r="A229" s="44">
         <v>228</v>
       </c>
@@ -64495,7 +64496,7 @@
       <c r="N229" s="29"/>
       <c r="O229" s="48"/>
     </row>
-    <row r="230" spans="1:15">
+    <row r="230" spans="1:15" hidden="1">
       <c r="A230" s="44">
         <v>229</v>
       </c>
@@ -64533,7 +64534,7 @@
       <c r="N230" s="29"/>
       <c r="O230" s="48"/>
     </row>
-    <row r="231" spans="1:15">
+    <row r="231" spans="1:15" hidden="1">
       <c r="A231" s="44">
         <v>230</v>
       </c>
@@ -64571,7 +64572,7 @@
       <c r="N231" s="29"/>
       <c r="O231" s="48"/>
     </row>
-    <row r="232" spans="1:15">
+    <row r="232" spans="1:15" hidden="1">
       <c r="A232" s="44">
         <v>231</v>
       </c>
@@ -64609,7 +64610,7 @@
       <c r="N232" s="29"/>
       <c r="O232" s="48"/>
     </row>
-    <row r="233" spans="1:15">
+    <row r="233" spans="1:15" hidden="1">
       <c r="A233" s="44">
         <v>232</v>
       </c>
@@ -64647,7 +64648,7 @@
       <c r="N233" s="29"/>
       <c r="O233" s="48"/>
     </row>
-    <row r="234" spans="1:15">
+    <row r="234" spans="1:15" hidden="1">
       <c r="A234" s="44">
         <v>233</v>
       </c>
@@ -64685,7 +64686,7 @@
       <c r="N234" s="29"/>
       <c r="O234" s="48"/>
     </row>
-    <row r="235" spans="1:15">
+    <row r="235" spans="1:15" hidden="1">
       <c r="A235" s="44">
         <v>234</v>
       </c>
@@ -64723,7 +64724,7 @@
       <c r="N235" s="29"/>
       <c r="O235" s="48"/>
     </row>
-    <row r="236" spans="1:15">
+    <row r="236" spans="1:15" hidden="1">
       <c r="A236" s="44">
         <v>235</v>
       </c>
@@ -64761,7 +64762,7 @@
       <c r="N236" s="29"/>
       <c r="O236" s="48"/>
     </row>
-    <row r="237" spans="1:15">
+    <row r="237" spans="1:15" hidden="1">
       <c r="A237" s="44">
         <v>236</v>
       </c>
@@ -64799,7 +64800,7 @@
       <c r="N237" s="29"/>
       <c r="O237" s="48"/>
     </row>
-    <row r="238" spans="1:15">
+    <row r="238" spans="1:15" hidden="1">
       <c r="A238" s="44">
         <v>237</v>
       </c>
@@ -64837,7 +64838,7 @@
       <c r="N238" s="29"/>
       <c r="O238" s="48"/>
     </row>
-    <row r="239" spans="1:15">
+    <row r="239" spans="1:15" hidden="1">
       <c r="A239" s="44">
         <v>238</v>
       </c>
@@ -64875,7 +64876,7 @@
       <c r="N239" s="29"/>
       <c r="O239" s="48"/>
     </row>
-    <row r="240" spans="1:15">
+    <row r="240" spans="1:15" hidden="1">
       <c r="A240" s="44">
         <v>239</v>
       </c>
@@ -64913,7 +64914,7 @@
       <c r="N240" s="29"/>
       <c r="O240" s="48"/>
     </row>
-    <row r="241" spans="1:15">
+    <row r="241" spans="1:15" hidden="1">
       <c r="A241" s="44">
         <v>240</v>
       </c>
@@ -64951,7 +64952,7 @@
       <c r="N241" s="29"/>
       <c r="O241" s="48"/>
     </row>
-    <row r="242" spans="1:15">
+    <row r="242" spans="1:15" hidden="1">
       <c r="A242" s="44">
         <v>241</v>
       </c>
@@ -64989,7 +64990,7 @@
       <c r="N242" s="29"/>
       <c r="O242" s="48"/>
     </row>
-    <row r="243" spans="1:15">
+    <row r="243" spans="1:15" hidden="1">
       <c r="A243" s="44">
         <v>242</v>
       </c>
@@ -65027,7 +65028,7 @@
       <c r="N243" s="29"/>
       <c r="O243" s="48"/>
     </row>
-    <row r="244" spans="1:15">
+    <row r="244" spans="1:15" hidden="1">
       <c r="A244" s="44">
         <v>243</v>
       </c>
@@ -65065,7 +65066,7 @@
       <c r="N244" s="29"/>
       <c r="O244" s="48"/>
     </row>
-    <row r="245" spans="1:15">
+    <row r="245" spans="1:15" hidden="1">
       <c r="A245" s="44">
         <v>244</v>
       </c>
@@ -65103,7 +65104,7 @@
       <c r="N245" s="29"/>
       <c r="O245" s="48"/>
     </row>
-    <row r="246" spans="1:15">
+    <row r="246" spans="1:15" hidden="1">
       <c r="A246" s="44">
         <v>245</v>
       </c>
@@ -65141,7 +65142,7 @@
       <c r="N246" s="29"/>
       <c r="O246" s="48"/>
     </row>
-    <row r="247" spans="1:15">
+    <row r="247" spans="1:15" hidden="1">
       <c r="A247" s="44">
         <v>246</v>
       </c>
@@ -65179,7 +65180,7 @@
       <c r="N247" s="29"/>
       <c r="O247" s="48"/>
     </row>
-    <row r="248" spans="1:15">
+    <row r="248" spans="1:15" hidden="1">
       <c r="A248" s="44">
         <v>247</v>
       </c>
@@ -65217,7 +65218,7 @@
       <c r="N248" s="29"/>
       <c r="O248" s="48"/>
     </row>
-    <row r="249" spans="1:15">
+    <row r="249" spans="1:15" hidden="1">
       <c r="A249" s="44">
         <v>248</v>
       </c>
@@ -65255,7 +65256,7 @@
       <c r="N249" s="29"/>
       <c r="O249" s="48"/>
     </row>
-    <row r="250" spans="1:15">
+    <row r="250" spans="1:15" hidden="1">
       <c r="A250" s="44">
         <v>249</v>
       </c>
@@ -65293,7 +65294,7 @@
       <c r="N250" s="29"/>
       <c r="O250" s="48"/>
     </row>
-    <row r="251" spans="1:15">
+    <row r="251" spans="1:15" hidden="1">
       <c r="A251" s="44">
         <v>250</v>
       </c>
@@ -65331,7 +65332,7 @@
       <c r="N251" s="29"/>
       <c r="O251" s="48"/>
     </row>
-    <row r="252" spans="1:15">
+    <row r="252" spans="1:15" hidden="1">
       <c r="A252" s="44">
         <v>251</v>
       </c>
@@ -65369,7 +65370,7 @@
       <c r="N252" s="29"/>
       <c r="O252" s="48"/>
     </row>
-    <row r="253" spans="1:15">
+    <row r="253" spans="1:15" hidden="1">
       <c r="A253" s="44">
         <v>252</v>
       </c>
@@ -65407,7 +65408,7 @@
       <c r="N253" s="29"/>
       <c r="O253" s="48"/>
     </row>
-    <row r="254" spans="1:15">
+    <row r="254" spans="1:15" hidden="1">
       <c r="A254" s="44">
         <v>253</v>
       </c>
@@ -65445,7 +65446,7 @@
       <c r="N254" s="29"/>
       <c r="O254" s="48"/>
     </row>
-    <row r="255" spans="1:15">
+    <row r="255" spans="1:15" hidden="1">
       <c r="A255" s="44">
         <v>254</v>
       </c>
@@ -65483,7 +65484,7 @@
       <c r="N255" s="29"/>
       <c r="O255" s="48"/>
     </row>
-    <row r="256" spans="1:15">
+    <row r="256" spans="1:15" hidden="1">
       <c r="A256" s="44">
         <v>255</v>
       </c>
@@ -65515,7 +65516,7 @@
       <c r="N256" s="29"/>
       <c r="O256" s="48"/>
     </row>
-    <row r="257" spans="1:15">
+    <row r="257" spans="1:15" hidden="1">
       <c r="A257" s="44">
         <v>256</v>
       </c>
@@ -65547,7 +65548,7 @@
       <c r="N257" s="29"/>
       <c r="O257" s="48"/>
     </row>
-    <row r="258" spans="1:15">
+    <row r="258" spans="1:15" hidden="1">
       <c r="A258" s="44">
         <v>257</v>
       </c>
@@ -65579,7 +65580,7 @@
       <c r="N258" s="29"/>
       <c r="O258" s="48"/>
     </row>
-    <row r="259" spans="1:15">
+    <row r="259" spans="1:15" hidden="1">
       <c r="A259" s="44">
         <v>258</v>
       </c>
@@ -65611,7 +65612,7 @@
       <c r="N259" s="29"/>
       <c r="O259" s="48"/>
     </row>
-    <row r="260" spans="1:15">
+    <row r="260" spans="1:15" hidden="1">
       <c r="A260" s="44">
         <v>259</v>
       </c>
@@ -65643,7 +65644,7 @@
       <c r="N260" s="29"/>
       <c r="O260" s="48"/>
     </row>
-    <row r="261" spans="1:15">
+    <row r="261" spans="1:15" hidden="1">
       <c r="A261" s="44">
         <v>260</v>
       </c>
@@ -65675,7 +65676,7 @@
       <c r="N261" s="29"/>
       <c r="O261" s="48"/>
     </row>
-    <row r="262" spans="1:15">
+    <row r="262" spans="1:15" hidden="1">
       <c r="A262" s="44">
         <v>261</v>
       </c>
@@ -65707,7 +65708,7 @@
       <c r="N262" s="29"/>
       <c r="O262" s="48"/>
     </row>
-    <row r="263" spans="1:15">
+    <row r="263" spans="1:15" hidden="1">
       <c r="A263" s="44">
         <v>262</v>
       </c>
@@ -65739,7 +65740,7 @@
       <c r="N263" s="29"/>
       <c r="O263" s="48"/>
     </row>
-    <row r="264" spans="1:15">
+    <row r="264" spans="1:15" hidden="1">
       <c r="A264" s="44">
         <v>263</v>
       </c>
@@ -65771,7 +65772,7 @@
       <c r="N264" s="29"/>
       <c r="O264" s="48"/>
     </row>
-    <row r="265" spans="1:15">
+    <row r="265" spans="1:15" hidden="1">
       <c r="A265" s="44">
         <v>264</v>
       </c>
@@ -65803,7 +65804,7 @@
       <c r="N265" s="29"/>
       <c r="O265" s="48"/>
     </row>
-    <row r="266" spans="1:15">
+    <row r="266" spans="1:15" hidden="1">
       <c r="A266" s="44">
         <v>265</v>
       </c>
@@ -65835,7 +65836,7 @@
       <c r="N266" s="29"/>
       <c r="O266" s="48"/>
     </row>
-    <row r="267" spans="1:15">
+    <row r="267" spans="1:15" hidden="1">
       <c r="A267" s="44">
         <v>266</v>
       </c>
@@ -65867,7 +65868,7 @@
       <c r="N267" s="29"/>
       <c r="O267" s="48"/>
     </row>
-    <row r="268" spans="1:15">
+    <row r="268" spans="1:15" hidden="1">
       <c r="A268" s="44">
         <v>267</v>
       </c>
@@ -65899,7 +65900,7 @@
       <c r="N268" s="29"/>
       <c r="O268" s="48"/>
     </row>
-    <row r="269" spans="1:15">
+    <row r="269" spans="1:15" hidden="1">
       <c r="A269" s="46">
         <v>268</v>
       </c>
@@ -66070,7 +66071,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O269" xr:uid="{A28DBFC5-8611-0B45-8E7C-1B1F27A6DFE8}"/>
+  <autoFilter ref="A1:O269" xr:uid="{A28DBFC5-8611-0B45-8E7C-1B1F27A6DFE8}">
+    <filterColumn colId="11">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>